<commit_message>
Test executions and .md files
</commit_message>
<xml_diff>
--- a/Test_Plans/Test_Cases/Amazon_Login_TestCases.xlsx
+++ b/Test_Plans/Test_Cases/Amazon_Login_TestCases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\Personal Project\VFX\QA-Portfolio\Test_Plans\Test_Cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A17B2FA8-7243-484D-82DC-0E7DB0D3923E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1789833A-6F3C-430F-967C-61859C6C9805}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{6108ADF1-4541-4B84-B66C-487326DA37E4}"/>
   </bookViews>
@@ -237,9 +237,6 @@
     <t>Enter email exceeding allowed length</t>
   </si>
   <si>
-    <t>Validation displayed or input restricted</t>
-  </si>
-  <si>
     <t>Boundary</t>
   </si>
   <si>
@@ -400,6 +397,9 @@
   </si>
   <si>
     <t>User logged out successfully</t>
+  </si>
+  <si>
+    <t>Login fails with incorrect password.</t>
   </si>
 </sst>
 </file>
@@ -1107,7 +1107,7 @@
         <v>62</v>
       </c>
       <c r="B16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C16" t="s">
         <v>50</v>
@@ -1122,7 +1122,7 @@
         <v>69</v>
       </c>
       <c r="G16" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
@@ -1130,7 +1130,7 @@
         <v>63</v>
       </c>
       <c r="B17" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C17" t="s">
         <v>50</v>
@@ -1139,13 +1139,13 @@
         <v>44</v>
       </c>
       <c r="E17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G17" t="s">
-        <v>56</v>
+        <v>124</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
@@ -1153,7 +1153,7 @@
         <v>64</v>
       </c>
       <c r="B18" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C18" t="s">
         <v>39</v>
@@ -1162,13 +1162,13 @@
         <v>44</v>
       </c>
       <c r="E18" t="s">
+        <v>73</v>
+      </c>
+      <c r="F18" t="s">
         <v>74</v>
       </c>
-      <c r="F18" t="s">
+      <c r="G18" t="s">
         <v>75</v>
-      </c>
-      <c r="G18" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
@@ -1176,7 +1176,7 @@
         <v>65</v>
       </c>
       <c r="B19" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C19" t="s">
         <v>50</v>
@@ -1185,21 +1185,21 @@
         <v>44</v>
       </c>
       <c r="E19" t="s">
+        <v>77</v>
+      </c>
+      <c r="F19" t="s">
         <v>78</v>
       </c>
-      <c r="F19" t="s">
+      <c r="G19" t="s">
         <v>79</v>
-      </c>
-      <c r="G19" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B20" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C20" t="s">
         <v>50</v>
@@ -1208,21 +1208,21 @@
         <v>44</v>
       </c>
       <c r="E20" t="s">
+        <v>81</v>
+      </c>
+      <c r="F20" t="s">
         <v>82</v>
       </c>
-      <c r="F20" t="s">
+      <c r="G20" t="s">
         <v>83</v>
-      </c>
-      <c r="G20" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B21" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C21" t="s">
         <v>50</v>
@@ -1231,21 +1231,21 @@
         <v>44</v>
       </c>
       <c r="E21" t="s">
+        <v>92</v>
+      </c>
+      <c r="F21" t="s">
         <v>93</v>
       </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
         <v>94</v>
-      </c>
-      <c r="G21" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B22" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C22" t="s">
         <v>50</v>
@@ -1254,21 +1254,21 @@
         <v>44</v>
       </c>
       <c r="E22" t="s">
+        <v>95</v>
+      </c>
+      <c r="F22" t="s">
         <v>96</v>
       </c>
-      <c r="F22" t="s">
+      <c r="G22" t="s">
         <v>97</v>
-      </c>
-      <c r="G22" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B23" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C23" t="s">
         <v>50</v>
@@ -1277,90 +1277,90 @@
         <v>44</v>
       </c>
       <c r="E23" t="s">
+        <v>98</v>
+      </c>
+      <c r="F23" t="s">
         <v>99</v>
       </c>
-      <c r="F23" t="s">
+      <c r="G23" t="s">
         <v>100</v>
-      </c>
-      <c r="G23" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B24" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C24" t="s">
         <v>50</v>
       </c>
       <c r="D24" t="s">
+        <v>103</v>
+      </c>
+      <c r="E24" t="s">
+        <v>102</v>
+      </c>
+      <c r="F24" t="s">
         <v>104</v>
       </c>
-      <c r="E24" t="s">
-        <v>103</v>
-      </c>
-      <c r="F24" t="s">
+      <c r="G24" t="s">
         <v>105</v>
-      </c>
-      <c r="G24" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B25" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C25" t="s">
         <v>50</v>
       </c>
       <c r="D25" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E25" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F25" t="s">
+        <v>104</v>
+      </c>
+      <c r="G25" t="s">
         <v>105</v>
-      </c>
-      <c r="G25" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B26" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C26" t="s">
         <v>50</v>
       </c>
       <c r="D26" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E26" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F26" t="s">
+        <v>104</v>
+      </c>
+      <c r="G26" t="s">
         <v>105</v>
-      </c>
-      <c r="G26" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B27" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C27" t="s">
         <v>39</v>
@@ -1369,59 +1369,59 @@
         <v>41</v>
       </c>
       <c r="E27" t="s">
+        <v>111</v>
+      </c>
+      <c r="F27" t="s">
         <v>112</v>
       </c>
-      <c r="F27" t="s">
+      <c r="G27" t="s">
         <v>113</v>
-      </c>
-      <c r="G27" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B28" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C28" t="s">
         <v>39</v>
       </c>
       <c r="D28" t="s">
+        <v>116</v>
+      </c>
+      <c r="E28" t="s">
+        <v>115</v>
+      </c>
+      <c r="F28" t="s">
         <v>117</v>
       </c>
-      <c r="E28" t="s">
-        <v>116</v>
-      </c>
-      <c r="F28" t="s">
+      <c r="G28" t="s">
         <v>118</v>
-      </c>
-      <c r="G28" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B29" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C29" t="s">
         <v>39</v>
       </c>
       <c r="D29" t="s">
+        <v>121</v>
+      </c>
+      <c r="E29" t="s">
+        <v>80</v>
+      </c>
+      <c r="F29" t="s">
         <v>122</v>
       </c>
-      <c r="E29" t="s">
-        <v>81</v>
-      </c>
-      <c r="F29" t="s">
+      <c r="G29" t="s">
         <v>123</v>
-      </c>
-      <c r="G29" t="s">
-        <v>124</v>
       </c>
     </row>
   </sheetData>

</xml_diff>